<commit_message>
add some space, relevant courses, hardware focus?
</commit_message>
<xml_diff>
--- a/omsas gpa calculator.xlsx
+++ b/omsas gpa calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/randyzhu/Desktop/resume/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72E176F2-24F3-7C46-A2D1-BACBA98C6523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{097BD9C5-6F30-3A4B-9FDC-F5DDFCC76002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18000" yWindow="780" windowWidth="18000" windowHeight="22600" xr2:uid="{D17FC236-BBBD-6343-BC06-859C4F9877D0}"/>
+    <workbookView xWindow="26560" yWindow="7140" windowWidth="18000" windowHeight="22600" xr2:uid="{D17FC236-BBBD-6343-BC06-859C4F9877D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="40">
   <si>
     <t>Grade</t>
   </si>
@@ -154,6 +154,12 @@
   </si>
   <si>
     <t>GPA</t>
+  </si>
+  <si>
+    <t>PHYS 131</t>
+  </si>
+  <si>
+    <t>D</t>
   </si>
 </sst>
 </file>
@@ -526,7 +532,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F82280FC-726A-9643-8ECE-C451CE42BB28}">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="6" max="6" width="10.83203125" style="1"/>
@@ -575,7 +581,7 @@
       </c>
       <c r="F2" s="1">
         <f>SUM(E:E)/SUM(C:C)</f>
-        <v>3.8461538461538463</v>
+        <v>3.8058823529411767</v>
       </c>
       <c r="G2" t="s">
         <v>3</v>
@@ -595,11 +601,11 @@
         <v>4</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D16" si="0">_xlfn.XLOOKUP(B3,G:G,H:H)</f>
+        <f t="shared" ref="D3:D22" si="0">_xlfn.XLOOKUP(B3,G:G,H:H)</f>
         <v>4</v>
       </c>
       <c r="E3">
-        <f t="shared" ref="E3:E16" si="1">C3*D3</f>
+        <f t="shared" ref="E3:E22" si="1">C3*D3</f>
         <v>16</v>
       </c>
       <c r="G3" t="s">
@@ -828,7 +834,7 @@
         <v>12</v>
       </c>
       <c r="G12" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -922,33 +928,123 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18">
+        <v>3</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="0"/>
+        <v>3.7</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="1"/>
+        <v>11.100000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19">
+        <v>3</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>2</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="0"/>
+        <v>3.9</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="1"/>
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>26</v>
       </c>
+      <c r="B21" t="s">
+        <v>2</v>
+      </c>
+      <c r="C21">
+        <v>3</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="0"/>
+        <v>3.9</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="1"/>
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22">
+        <f t="shared" si="0"/>
+        <v>2.7</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="1"/>
+        <v>8.1000000000000014</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>